<commit_message>
feat/ sku + renombrar presentacion fix
</commit_message>
<xml_diff>
--- a/scripts/files/import-tango-gamas.xlsx
+++ b/scripts/files/import-tango-gamas.xlsx
@@ -5549,21 +5549,21 @@
     </row>
     <row r="435" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A435">
-        <v>176</v>
+        <v>327</v>
       </c>
       <c r="B435" t="s">
-        <v>42</v>
+        <v>3</v>
       </c>
       <c r="C435" t="s">
-        <v>9</v>
+        <v>6</v>
       </c>
     </row>
     <row r="436" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A436">
-        <v>316</v>
+        <v>327</v>
       </c>
       <c r="B436" t="s">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="C436" t="s">
         <v>4</v>
@@ -5571,21 +5571,21 @@
     </row>
     <row r="437" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A437">
-        <v>164</v>
+        <v>327</v>
       </c>
       <c r="B437" t="s">
-        <v>26</v>
+        <v>7</v>
       </c>
       <c r="C437" t="s">
-        <v>9</v>
+        <v>6</v>
       </c>
     </row>
     <row r="438" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A438">
-        <v>164</v>
+        <v>176</v>
       </c>
       <c r="B438" t="s">
-        <v>27</v>
+        <v>42</v>
       </c>
       <c r="C438" t="s">
         <v>9</v>
@@ -5593,46 +5593,46 @@
     </row>
     <row r="439" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A439">
-        <v>164</v>
+        <v>316</v>
       </c>
       <c r="B439" t="s">
-        <v>28</v>
+        <v>3</v>
       </c>
       <c r="C439" t="s">
-        <v>9</v>
+        <v>4</v>
       </c>
     </row>
     <row r="440" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A440">
-        <v>59</v>
+        <v>164</v>
       </c>
       <c r="B440" t="s">
-        <v>7</v>
+        <v>26</v>
       </c>
       <c r="C440" t="s">
-        <v>17</v>
+        <v>9</v>
       </c>
     </row>
     <row r="441" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A441">
-        <v>59</v>
+        <v>164</v>
       </c>
       <c r="B441" t="s">
-        <v>14</v>
+        <v>27</v>
       </c>
       <c r="C441" t="s">
-        <v>6</v>
+        <v>9</v>
       </c>
     </row>
     <row r="442" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A442">
-        <v>59</v>
+        <v>164</v>
       </c>
       <c r="B442" t="s">
-        <v>12</v>
+        <v>28</v>
       </c>
       <c r="C442" t="s">
-        <v>6</v>
+        <v>9</v>
       </c>
     </row>
     <row r="443" spans="1:3" x14ac:dyDescent="0.25">
@@ -5640,7 +5640,7 @@
         <v>59</v>
       </c>
       <c r="B443" t="s">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="C443" t="s">
         <v>17</v>
@@ -5651,43 +5651,43 @@
         <v>59</v>
       </c>
       <c r="B444" t="s">
-        <v>3</v>
+        <v>14</v>
       </c>
       <c r="C444" t="s">
-        <v>17</v>
+        <v>6</v>
       </c>
     </row>
     <row r="445" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A445">
-        <v>317</v>
+        <v>59</v>
       </c>
       <c r="B445" t="s">
-        <v>3</v>
+        <v>12</v>
       </c>
       <c r="C445" t="s">
-        <v>4</v>
+        <v>6</v>
       </c>
     </row>
     <row r="446" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A446">
-        <v>317</v>
+        <v>59</v>
       </c>
       <c r="B446" t="s">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="C446" t="s">
-        <v>4</v>
+        <v>17</v>
       </c>
     </row>
     <row r="447" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A447">
-        <v>317</v>
+        <v>59</v>
       </c>
       <c r="B447" t="s">
-        <v>43</v>
+        <v>3</v>
       </c>
       <c r="C447" t="s">
-        <v>4</v>
+        <v>17</v>
       </c>
     </row>
     <row r="448" spans="1:3" x14ac:dyDescent="0.25">
@@ -5695,7 +5695,7 @@
         <v>317</v>
       </c>
       <c r="B448" t="s">
-        <v>14</v>
+        <v>3</v>
       </c>
       <c r="C448" t="s">
         <v>4</v>
@@ -5703,10 +5703,10 @@
     </row>
     <row r="449" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A449">
-        <v>318</v>
+        <v>317</v>
       </c>
       <c r="B449" t="s">
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="C449" t="s">
         <v>4</v>
@@ -5714,10 +5714,10 @@
     </row>
     <row r="450" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A450">
-        <v>319</v>
+        <v>317</v>
       </c>
       <c r="B450" t="s">
-        <v>3</v>
+        <v>43</v>
       </c>
       <c r="C450" t="s">
         <v>4</v>
@@ -5725,10 +5725,10 @@
     </row>
     <row r="451" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A451">
-        <v>123</v>
+        <v>317</v>
       </c>
       <c r="B451" t="s">
-        <v>3</v>
+        <v>14</v>
       </c>
       <c r="C451" t="s">
         <v>4</v>
@@ -5736,10 +5736,10 @@
     </row>
     <row r="452" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A452">
-        <v>123</v>
+        <v>318</v>
       </c>
       <c r="B452" t="s">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="C452" t="s">
         <v>4</v>
@@ -5747,10 +5747,10 @@
     </row>
     <row r="453" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A453">
-        <v>123</v>
+        <v>319</v>
       </c>
       <c r="B453" t="s">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="C453" t="s">
         <v>4</v>
@@ -5761,7 +5761,7 @@
         <v>123</v>
       </c>
       <c r="B454" t="s">
-        <v>19</v>
+        <v>3</v>
       </c>
       <c r="C454" t="s">
         <v>4</v>
@@ -5769,32 +5769,32 @@
     </row>
     <row r="455" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A455">
-        <v>320</v>
+        <v>123</v>
       </c>
       <c r="B455" t="s">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="C455" t="s">
-        <v>6</v>
+        <v>4</v>
       </c>
     </row>
     <row r="456" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A456">
-        <v>320</v>
+        <v>123</v>
       </c>
       <c r="B456" t="s">
         <v>7</v>
       </c>
       <c r="C456" t="s">
-        <v>6</v>
+        <v>4</v>
       </c>
     </row>
     <row r="457" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A457">
-        <v>321</v>
+        <v>123</v>
       </c>
       <c r="B457" t="s">
-        <v>3</v>
+        <v>19</v>
       </c>
       <c r="C457" t="s">
         <v>4</v>
@@ -5802,18 +5802,18 @@
     </row>
     <row r="458" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A458">
-        <v>322</v>
+        <v>320</v>
       </c>
       <c r="B458" t="s">
         <v>3</v>
       </c>
       <c r="C458" t="s">
-        <v>4</v>
+        <v>6</v>
       </c>
     </row>
     <row r="459" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A459">
-        <v>322</v>
+        <v>320</v>
       </c>
       <c r="B459" t="s">
         <v>7</v>
@@ -5824,7 +5824,7 @@
     </row>
     <row r="460" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A460">
-        <v>323</v>
+        <v>321</v>
       </c>
       <c r="B460" t="s">
         <v>3</v>
@@ -5835,10 +5835,10 @@
     </row>
     <row r="461" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A461">
-        <v>323</v>
+        <v>322</v>
       </c>
       <c r="B461" t="s">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="C461" t="s">
         <v>4</v>
@@ -5846,13 +5846,13 @@
     </row>
     <row r="462" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A462">
-        <v>323</v>
+        <v>322</v>
       </c>
       <c r="B462" t="s">
-        <v>12</v>
+        <v>7</v>
       </c>
       <c r="C462" t="s">
-        <v>4</v>
+        <v>6</v>
       </c>
     </row>
     <row r="463" spans="1:3" x14ac:dyDescent="0.25">
@@ -5860,7 +5860,7 @@
         <v>323</v>
       </c>
       <c r="B463" t="s">
-        <v>14</v>
+        <v>3</v>
       </c>
       <c r="C463" t="s">
         <v>4</v>
@@ -5868,21 +5868,21 @@
     </row>
     <row r="464" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A464">
-        <v>324</v>
+        <v>323</v>
       </c>
       <c r="B464" t="s">
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="C464" t="s">
-        <v>17</v>
+        <v>4</v>
       </c>
     </row>
     <row r="465" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A465">
-        <v>324</v>
+        <v>323</v>
       </c>
       <c r="B465" t="s">
-        <v>5</v>
+        <v>12</v>
       </c>
       <c r="C465" t="s">
         <v>4</v>
@@ -5890,13 +5890,13 @@
     </row>
     <row r="466" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A466">
-        <v>324</v>
+        <v>323</v>
       </c>
       <c r="B466" t="s">
-        <v>7</v>
+        <v>14</v>
       </c>
       <c r="C466" t="s">
-        <v>17</v>
+        <v>4</v>
       </c>
     </row>
     <row r="467" spans="1:3" x14ac:dyDescent="0.25">
@@ -5904,51 +5904,51 @@
         <v>324</v>
       </c>
       <c r="B467" t="s">
-        <v>14</v>
+        <v>3</v>
       </c>
       <c r="C467" t="s">
-        <v>4</v>
+        <v>17</v>
       </c>
     </row>
     <row r="468" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A468">
-        <v>325</v>
+        <v>324</v>
       </c>
       <c r="B468" t="s">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="C468" t="s">
-        <v>6</v>
+        <v>4</v>
       </c>
     </row>
     <row r="469" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A469">
-        <v>325</v>
+        <v>324</v>
       </c>
       <c r="B469" t="s">
         <v>7</v>
       </c>
       <c r="C469" t="s">
-        <v>6</v>
+        <v>17</v>
       </c>
     </row>
     <row r="470" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A470">
-        <v>326</v>
+        <v>324</v>
       </c>
       <c r="B470" t="s">
-        <v>3</v>
+        <v>14</v>
       </c>
       <c r="C470" t="s">
-        <v>6</v>
+        <v>4</v>
       </c>
     </row>
     <row r="471" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A471">
-        <v>326</v>
+        <v>325</v>
       </c>
       <c r="B471" t="s">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="C471" t="s">
         <v>6</v>
@@ -5956,7 +5956,7 @@
     </row>
     <row r="472" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A472">
-        <v>326</v>
+        <v>325</v>
       </c>
       <c r="B472" t="s">
         <v>7</v>
@@ -5970,7 +5970,7 @@
         <v>326</v>
       </c>
       <c r="B473" t="s">
-        <v>14</v>
+        <v>3</v>
       </c>
       <c r="C473" t="s">
         <v>6</v>
@@ -5978,10 +5978,10 @@
     </row>
     <row r="474" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A474">
-        <v>327</v>
+        <v>326</v>
       </c>
       <c r="B474" t="s">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="C474" t="s">
         <v>6</v>
@@ -5989,21 +5989,21 @@
     </row>
     <row r="475" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A475">
-        <v>327</v>
+        <v>326</v>
       </c>
       <c r="B475" t="s">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="C475" t="s">
-        <v>4</v>
+        <v>6</v>
       </c>
     </row>
     <row r="476" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A476">
-        <v>327</v>
+        <v>326</v>
       </c>
       <c r="B476" t="s">
-        <v>7</v>
+        <v>14</v>
       </c>
       <c r="C476" t="s">
         <v>6</v>

</xml_diff>